<commit_message>
ops(vevor): generate shared full feed and worker packet
</commit_message>
<xml_diff>
--- a/operations/vendor-source/vevor/2026-09-10/04_Elevation_VEVOR_Curated_Catalog_Working_Set_2026-09-10_PUBLIC_SAFE.xlsx
+++ b/operations/vendor-source/vevor/2026-09-10/04_Elevation_VEVOR_Curated_Catalog_Working_Set_2026-09-10_PUBLIC_SAFE.xlsx
@@ -537,7 +537,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>384</t>
+          <t>381</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -609,7 +609,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>126</t>
+          <t>125</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -681,7 +681,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>216</t>
+          <t>209</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -825,7 +825,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>491</t>
+          <t>488</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -897,7 +897,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>289</t>
+          <t>287</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -969,7 +969,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>159</t>
+          <t>158</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -1041,7 +1041,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>15563</t>
+          <t>16908</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -1113,7 +1113,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>321</t>
+          <t>315</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -1185,7 +1185,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2916</t>
+          <t>2904</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1257,7 +1257,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2551</t>
+          <t>2546</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1401,7 +1401,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>160</t>
+          <t>157</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1689,7 +1689,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>8557</t>
+          <t>8545</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -1761,7 +1761,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>9910</t>
+          <t>9898</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -1833,7 +1833,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>2462</t>
+          <t>2451</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -1905,7 +1905,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>486</t>
+          <t>484</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -1977,7 +1977,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>595</t>
+          <t>592</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -2049,7 +2049,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>402</t>
+          <t>400</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -2121,7 +2121,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>1514</t>
+          <t>1509</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -2193,7 +2193,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>13178</t>
+          <t>13141</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -2265,7 +2265,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>2416</t>
+          <t>2398</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -2337,7 +2337,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>131</t>
+          <t>128</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -2409,7 +2409,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>1140</t>
+          <t>1137</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -2481,7 +2481,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>564</t>
+          <t>562</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -2553,7 +2553,7 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>560</t>
+          <t>550</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -2697,7 +2697,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>1919</t>
+          <t>1917</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -2769,7 +2769,7 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>1779</t>
+          <t>1757</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -2841,7 +2841,7 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>2684</t>
+          <t>2672</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
@@ -2913,7 +2913,7 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>3086</t>
+          <t>3072</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -2985,7 +2985,7 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>1640</t>
+          <t>1634</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -3057,7 +3057,7 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>899</t>
+          <t>894</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -3129,7 +3129,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>1991</t>
+          <t>1975</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -3201,7 +3201,7 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>2885</t>
+          <t>2876</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
@@ -3273,7 +3273,7 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>310</t>
+          <t>303</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
@@ -3345,7 +3345,7 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>49</t>
+          <t>48</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
@@ -3501,7 +3501,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>20993</v>
+        <v>21005</v>
       </c>
     </row>
     <row r="4">
@@ -3511,7 +3511,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>16023</v>
+        <v>16038</v>
       </c>
     </row>
     <row r="5">

</xml_diff>

<commit_message>
ops(vevor): generate shared full feed and worker assets
</commit_message>
<xml_diff>
--- a/operations/vendor-source/vevor/2026-09-10/04_Elevation_VEVOR_Curated_Catalog_Working_Set_2026-09-10_PUBLIC_SAFE.xlsx
+++ b/operations/vendor-source/vevor/2026-09-10/04_Elevation_VEVOR_Curated_Catalog_Working_Set_2026-09-10_PUBLIC_SAFE.xlsx
@@ -537,7 +537,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>381</t>
+          <t>395</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -609,7 +609,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>125</t>
+          <t>143</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -681,7 +681,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>209</t>
+          <t>206</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -825,7 +825,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>488</t>
+          <t>485</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -897,7 +897,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>287</t>
+          <t>286</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -969,7 +969,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>158</t>
+          <t>157</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -1041,7 +1041,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>16908</t>
+          <t>17519</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -1185,7 +1185,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2904</t>
+          <t>2895</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1257,7 +1257,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2546</t>
+          <t>2533</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1401,7 +1401,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>157</t>
+          <t>153</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -1473,7 +1473,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>191</t>
+          <t>189</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1545,7 +1545,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>141</t>
+          <t>140</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -1689,7 +1689,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>8545</t>
+          <t>8536</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -1761,7 +1761,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>9898</t>
+          <t>10313</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -1833,7 +1833,7 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>2451</t>
+          <t>2444</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -1905,7 +1905,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>484</t>
+          <t>483</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -1977,7 +1977,7 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>592</t>
+          <t>589</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -2049,7 +2049,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>400</t>
+          <t>399</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -2121,7 +2121,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>1509</t>
+          <t>1498</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -2193,7 +2193,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>13141</t>
+          <t>13125</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -2265,7 +2265,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>2398</t>
+          <t>2388</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -2337,7 +2337,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>128</t>
+          <t>142</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -2409,7 +2409,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>1137</t>
+          <t>1132</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -2481,7 +2481,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>562</t>
+          <t>561</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -2553,7 +2553,7 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>550</t>
+          <t>529</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -2625,7 +2625,7 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>880</t>
+          <t>878</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
@@ -2697,7 +2697,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>1917</t>
+          <t>1915</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -2769,7 +2769,7 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>1757</t>
+          <t>1734</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -2841,7 +2841,7 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>2672</t>
+          <t>2680</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
@@ -2913,7 +2913,7 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>3072</t>
+          <t>3061</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -2985,7 +2985,7 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>1634</t>
+          <t>1632</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -3057,7 +3057,7 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>894</t>
+          <t>885</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -3129,7 +3129,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>1975</t>
+          <t>2045</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -3201,7 +3201,7 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>2876</t>
+          <t>2870</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
@@ -3273,7 +3273,7 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>303</t>
+          <t>302</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
@@ -3345,7 +3345,7 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>48</t>
+          <t>50</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
@@ -3511,7 +3511,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>16038</v>
+        <v>16011</v>
       </c>
     </row>
     <row r="5">

</xml_diff>